<commit_message>
feat(catalogo): indice central de productos (un producto = un sitio)
- data/catalogo.json: 154 productos agrupados por ASIN, 17 compartidos en 2+ kits
- scripts/catalogo.py: build | donde | compartidos | huecos | sustituir | verificar
  (sustituir arregla un ASIN muerto en TODOS los kits de una pasada: el bug de la manta)
- 154/154 fichas verificadas vivas; buscador nocturno aplico 3 fichas nuevas
- nota con el diseno y las reglas
</commit_message>
<xml_diff>
--- a/data/productos-pendientes.xlsx
+++ b/data/productos-pendientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pendientes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pendientes'!$A$1:$L$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pendientes'!$A$1:$L$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1024,20 +1024,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>kit-hogar</t>
+          <t>kit-evacuacion</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Luz, energía y comunicación</t>
+          <t>Utilidad</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Radio FM/AM a pilas o de dinamo</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Efectivo en billetes pequeños</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>efectivo en billetes pequeños</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -1045,7 +1049,7 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -1056,20 +1060,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>kit-hogar</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Luz, energía y comunicación</t>
+          <t>Para empezar a sembrar</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Batería externa (powerbank) de 10.000-20.000 mAh</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>Medidor de humedad y pH del suelo (3-en-1)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.amazon.es/s?k=medidor+humedad+ph+suelo&amp;tag=nti0c8-21</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -1077,7 +1085,7 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1088,22 +1096,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>kit-evacuacion</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Utilidad</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Efectivo en billetes pequeños</t>
+          <t>Compostera doméstica con grifo (20 L)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>efectivo en billetes pequeños</t>
+          <t>https://www.amazon.es/s?k=compostera+domestica+20l+grifo&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1113,7 +1121,7 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>N/A — no es compra online</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -1124,22 +1132,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>kit-evacuacion</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Utilidad</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Elemento luminoso o reflectante para caminar de noche (obligatorio para peatones)</t>
+          <t>Malla anti-áfidos invernadero (2 x 8 m, 30 mesh)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>chaleco reflectante peaton luminoso</t>
+          <t>https://www.amazon.es/s?k=malla+anti+afidos+invernadero+2x8&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1149,7 +1157,7 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -1165,17 +1173,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Para empezar a sembrar</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Medidor de humedad y pH del suelo (3-en-1)</t>
+          <t>Kit riego por goteo básico (10-20 plantas)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=medidor+humedad+ph+suelo&amp;tag=nti0c8-21</t>
+          <t>https://www.amazon.es/s?k=riego+goteo+jardin+kit+plantas&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1206,12 +1214,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Compostera doméstica con grifo (20 L)</t>
+          <t>Red antipájaros para huerto (1x3 m, malla fina 2 cm)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=compostera+domestica+20l+grifo&amp;tag=nti0c8-21</t>
+          <t>https://www.amazon.es/s?k=red+antipajaros+huerto+1x3&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1232,22 +1240,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-30-dias</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Agua (180 L para 2 personas / 30 días)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Malla anti-áfidos invernadero (2 x 8 m, 30 mesh)</t>
+          <t>Renueva el agua cada 6 meses</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=malla+anti+afidos+invernadero+2x8&amp;tag=nti0c8-21</t>
+          <t>renueva el agua cada 6 meses</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1257,7 +1265,7 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -1268,22 +1276,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Leche y comida de reserva</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kit riego por goteo básico (10-20 plantas)</t>
+          <t>Fórmula líquida lista para consumir (envases de 200 ml, pack de 6-12)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=riego+goteo+jardin+kit+plantas&amp;tag=nti0c8-21</t>
+          <t>https://www.amazon.es/s?k=formula+lactante+liquida+lista+para+consumir+200+ml&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -1304,22 +1312,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Higiene y pañales</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Red antipájaros para huerto (1x3 m, malla fina 2 cm)</t>
+          <t>Pastillas esterilizadoras en frío para biberones y tetinas</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=red+antipajaros+huerto+1x3&amp;tag=nti0c8-21</t>
+          <t>https://www.amazon.es/s?k=pastillas+esterilizadoras+biberones+agua+fria&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1340,22 +1348,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>kit-30-dias</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Agua (180 L para 2 personas / 30 días)</t>
+          <t>Abrigo y sueño</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Renueva el agua cada 6 meses</t>
+          <t>Cuna de viaje plegable (o capazo rígido de recién nacido)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>renueva el agua cada 6 meses</t>
+          <t>https://www.amazon.es/s?k=cuna+de+viaje+plegable+bebe&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -1365,7 +1373,7 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>N/A — no es compra online</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -1381,17 +1389,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Leche y comida de reserva</t>
+          <t>Salud y calma</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Fórmula líquida lista para consumir (envases de 200 ml, pack de 6-12)</t>
+          <t>Chupetes de reserva (2-3, la talla que usa ahora) y portachupete</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=formula+lactante+liquida+lista+para+consumir+200+ml&amp;tag=nti0c8-21</t>
+          <t>https://www.amazon.es/s?k=chupete+bebe+talla+por+edad&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1412,22 +1420,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>kit-bebe</t>
+          <t>kit-mayores</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Higiene y pañales</t>
+          <t>Comunicación y compañía</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Pastillas esterilizadoras en frío para biberones y tetinas</t>
+          <t>Hoja de contactos en papel con letra grande (112, familia, médico, vecino, farmacia)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=pastillas+esterilizadoras+biberones+agua+fria&amp;tag=nti0c8-21</t>
+          <t>hoja de contactos en papel con letra grande</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1448,22 +1456,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kit-bebe</t>
+          <t>kit-mayores</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Abrigo y sueño</t>
+          <t>Comunicación y compañía</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Cuna de viaje plegable (o capazo rígido de recién nacido)</t>
+          <t>Acuerdo de vecindad con llamada/golpe de aviso</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=cuna+de+viaje+plegable+bebe&amp;tag=nti0c8-21</t>
+          <t>acuerdo de vecindad con llamada golpe de aviso</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -1478,116 +1486,8 @@
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>kit-bebe</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Salud y calma</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Chupetes de reserva (2-3, la talla que usa ahora) y portachupete</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=chupete+bebe+talla+por+edad&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>sin candidato verificado</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>kit-mayores</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Comunicación y compañía</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Hoja de contactos en papel con letra grande (112, familia, médico, vecino, farmacia)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>hoja de contactos en papel con letra grande</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>sin candidato verificado</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>kit-mayores</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Comunicación y compañía</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Acuerdo de vecindad con llamada/golpe de aviso</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>acuerdo de vecindad con llamada golpe de aviso</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>sin candidato verificado</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L32"/>
+  <autoFilter ref="A1:L29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(seo): optimizar meta tags para CTR (5 mejoras)
</commit_message>
<xml_diff>
--- a/data/productos-pendientes.xlsx
+++ b/data/productos-pendientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendientes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pendientes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pendientes'!$A$1:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pendientes'!$A$1:$L$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -536,22 +536,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>kit-dana</t>
+          <t>kit-apagon</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Comunicación y avisos: cuando cae la red</t>
+          <t>Seguridad durante el corte</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Radio FM/AM a pilas o de manivela, con linterna integrada</t>
+          <t>Detector de monóxido de carbono (CO) a pilas con alarma</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>radio fm a pilas con dinamo y linterna</t>
+          <t>detector de monoxido de carbono co a pilas con alarma</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -572,22 +572,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>kit-dana</t>
+          <t>kit-apagon</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Comunicación y avisos: cuando cae la red</t>
+          <t>Seguridad durante el corte</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Walkie-talkies PMR446 (pareja con cargador)</t>
+          <t>Extintor de polvo ABC de 1-2 kg con soporte</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>walkie talkies pmr446 pareja recargables</t>
+          <t>extintor de polvo abc 1 kg con soporte pared</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -608,24 +608,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>kit-dana</t>
+          <t>kit-apagon</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Comunicación y avisos: cuando cae la red</t>
+          <t>Dinero y comunicación</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Batería externa (power bank) 10.000-20.000 mAh, dos salidas</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>bateria externa power bank 20000 mah dos salidas</t>
-        </is>
-      </c>
+          <t>Caja fuerte pequeña portátil para efectivo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -633,7 +629,7 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -644,22 +640,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>kit-dana</t>
+          <t>kit-hogar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Comunicación y avisos: cuando cae la red</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mascarilla FFP2 (pack) y gafas de protección para la limpieza</t>
+          <t>Paracetamol e ibuprofeno (caducidad larga)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>mascarilla ffp2 pack 10 gafas de proteccion</t>
+          <t>paracetamol e ibuprofeno</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -669,7 +665,7 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -680,22 +676,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>kit-apagon</t>
+          <t>kit-evacuacion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cocina sin electricidad</t>
+          <t>Utilidad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Acumuladores de frío (bloques de gel congelables) para nevera y congelador</t>
+          <t>Efectivo en billetes pequeños</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>acumulador de frio bloques de gel congelables nevera</t>
+          <t>efectivo en billetes pequeños</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -705,7 +701,7 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -716,22 +712,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>kit-apagon</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Seguridad durante el corte</t>
+          <t>Para empezar a sembrar</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Detector de monóxido de carbono (CO) a pilas con alarma</t>
+          <t>Medidor de humedad y pH del suelo (3-en-1)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>detector de monoxido de carbono co a pilas con alarma</t>
+          <t>https://www.amazon.es/s?k=medidor+humedad+ph+suelo&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -741,7 +737,7 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -752,22 +748,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>kit-apagon</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Seguridad durante el corte</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Extintor de polvo ABC de 1-2 kg con soporte</t>
+          <t>Compostera doméstica con grifo (20 L)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>extintor de polvo abc 1 kg con soporte pared</t>
+          <t>https://www.amazon.es/s?k=compostera+domestica+20l+grifo&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -777,7 +773,7 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -788,20 +784,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>kit-apagon</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dinero y comunicación</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Caja fuerte pequeña portátil para efectivo</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>Malla anti-áfidos invernadero (2 x 8 m, 30 mesh)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://www.amazon.es/s?k=malla+anti+afidos+invernadero+2x8&amp;tag=nti0c8-21</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -809,7 +809,7 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>N/A — no es compra online</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -820,22 +820,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>kit-apagon</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dinero y comunicación</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SAI / UPS pequeño (600-900 VA) para router y ONT</t>
+          <t>Kit riego por goteo básico (10-20 plantas)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sai ups 600va router ont bateria</t>
+          <t>https://www.amazon.es/s?k=riego+goteo+jardin+kit+plantas&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -845,7 +845,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -856,22 +856,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>kit-coche</t>
+          <t>huerto-autosuficiencia</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Obligatorio en España (DGT)</t>
+          <t>Compostaje y protección</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Chaleco reflectante de alta visibilidad (dotación obligatoria en moto)</t>
+          <t>Red antipájaros para huerto (1x3 m, malla fina 2 cm)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>chaleco reflectante alta visibilidad</t>
+          <t>https://www.amazon.es/s?k=red+antipajaros+huerto+1x3&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -881,7 +881,7 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -892,20 +892,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>kit-hogar</t>
+          <t>kit-30-dias</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cocina sin electricidad</t>
+          <t>Agua (180 L para 2 personas / 30 días)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Detector de monóxido de carbono a pilas</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Renueva el agua cada 6 meses</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>renueva el agua cada 6 meses</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -913,7 +917,7 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -924,22 +928,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>kit-hogar</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Leche y comida de reserva</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Paracetamol e ibuprofeno (caducidad larga)</t>
+          <t>Fórmula líquida lista para consumir (envases de 200 ml, pack de 6-12)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>paracetamol e ibuprofeno</t>
+          <t>https://www.amazon.es/s?k=formula+lactante+liquida+lista+para+consumir+200+ml&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -949,7 +953,7 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>N/A — no es compra online</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -960,20 +964,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>kit-hogar</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ventilación y calidad del aire</t>
+          <t>Higiene y pañales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Medidor de CO2 o calidad del aire portátil</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Pastillas esterilizadoras en frío para biberones y tetinas</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.amazon.es/s?k=pastillas+esterilizadoras+biberones+agua+fria&amp;tag=nti0c8-21</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -981,7 +989,7 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -992,20 +1000,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>kit-hogar</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Luz, energía y comunicación</t>
+          <t>Abrigo y sueño</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Linterna LED a pilas o de dinamo</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Cuna de viaje plegable (o capazo rígido de recién nacido)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.amazon.es/s?k=cuna+de+viaje+plegable+bebe&amp;tag=nti0c8-21</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -1013,7 +1025,7 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>propuesta</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -1024,22 +1036,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>kit-evacuacion</t>
+          <t>kit-bebe</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Utilidad</t>
+          <t>Salud y calma</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Efectivo en billetes pequeños</t>
+          <t>Chupetes de reserva (2-3, la talla que usa ahora) y portachupete</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>efectivo en billetes pequeños</t>
+          <t>https://www.amazon.es/s?k=chupete+bebe+talla+por+edad&amp;tag=nti0c8-21</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1049,7 +1061,7 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>N/A — no es compra online</t>
+          <t>sin candidato verificado</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -1060,22 +1072,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-mayores</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Para empezar a sembrar</t>
+          <t>Comunicación y compañía</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Medidor de humedad y pH del suelo (3-en-1)</t>
+          <t>Hoja de contactos en papel con letra grande (112, familia, médico, vecino, farmacia)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=medidor+humedad+ph+suelo&amp;tag=nti0c8-21</t>
+          <t>hoja de contactos en papel con letra grande</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1096,22 +1108,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-mayores</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Comunicación y compañía</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Compostera doméstica con grifo (20 L)</t>
+          <t>Acuerdo de vecindad con llamada/golpe de aviso</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://www.amazon.es/s?k=compostera+domestica+20l+grifo&amp;tag=nti0c8-21</t>
+          <t>acuerdo de vecindad con llamada golpe de aviso</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1132,24 +1144,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-frio</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Calor corporal: la capa que salva</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Malla anti-áfidos invernadero (2 x 8 m, 30 mesh)</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=malla+anti+afidos+invernadero+2x8&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Forro polar o jersey de lana</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -1168,24 +1176,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-terremoto</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Polvo, papeles y dinero</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kit riego por goteo básico (10-20 plantas)</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=riego+goteo+jardin+kit+plantas&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Efectivo en billetes pequeños</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -1193,7 +1197,7 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -1204,24 +1208,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>huerto-autosuficiencia</t>
+          <t>kit-incendio</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Compostaje y protección</t>
+          <t>Salir en 10 minutos</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Red antipájaros para huerto (1x3 m, malla fina 2 cm)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=red+antipajaros+huerto+1x3&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Carpeta estanca con documentos y algo de efectivo</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -1229,7 +1229,7 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>N/A — no es compra online</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -1240,24 +1240,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>kit-30-dias</t>
+          <t>kit-starlink</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Agua (180 L para 2 personas / 30 días)</t>
+          <t>Starlink: internet desde cualquier lugar</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Renueva el agua cada 6 meses</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>renueva el agua cada 6 meses</t>
-        </is>
-      </c>
+          <t>Cable extensor para Starlink (30 m / 60 m)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1265,7 +1261,7 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>N/A — no es compra online</t>
+          <t>propuesta</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -1276,24 +1272,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>kit-bebe</t>
+          <t>kit-starlink</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Leche y comida de reserva</t>
+          <t>Redundancia: router 4G/5G como respaldo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Fórmula líquida lista para consumir (envases de 200 ml, pack de 6-12)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=formula+lactante+liquida+lista+para+consumir+200+ml&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Router 4G/5G industrial con dual SIM y antenas externas</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1301,7 +1293,7 @@
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>propuesta</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -1312,24 +1304,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>kit-bebe</t>
+          <t>kit-starlink</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Higiene y pañales</t>
+          <t>Redundancia: router 4G/5G como respaldo</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Pastillas esterilizadoras en frío para biberones y tetinas</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=pastillas+esterilizadoras+biberones+agua+fria&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Antena externa 4G/5G de alta ganancia</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1337,7 +1325,7 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>propuesta</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -1348,24 +1336,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>kit-bebe</t>
+          <t>kit-starlink</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Abrigo y sueño</t>
+          <t>Último recurso: messenger satelital</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Cuna de viaje plegable (o capazo rígido de recién nacido)</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=cuna+de+viaje+plegable+bebe&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Messenger satelital (Garmin inReach Mini 3)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1373,7 +1357,7 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>propuesta</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -1384,24 +1368,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>kit-bebe</t>
+          <t>kit-kit-profesional</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Salud y calma</t>
+          <t>Energía solar: el sol es tu generador</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Chupetes de reserva (2-3, la talla que usa ahora) y portachupete</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://www.amazon.es/s?k=chupete+bebe+talla+por+edad&amp;tag=nti0c8-21</t>
-        </is>
-      </c>
+          <t>Panel solar 400W monocristalino (×2 unidades)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1409,7 +1389,7 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>propuesta</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
@@ -1420,24 +1400,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>kit-mayores</t>
+          <t>kit-kit-profesional</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Comunicación y compañía</t>
+          <t>Energía solar: el sol es tu generador</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Hoja de contactos en papel con letra grande (112, familia, médico, vecino, farmacia)</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>hoja de contactos en papel con letra grande</t>
-        </is>
-      </c>
+          <t>Inversor híbrido 3000W-5000W</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1445,7 +1421,7 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>sin candidato verificado</t>
+          <t>propuesta</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -1456,24 +1432,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>kit-mayores</t>
+          <t>kit-kit-profesional</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Comunicación y compañía</t>
+          <t>Energía solar: el sol es tu generador</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Acuerdo de vecindad con llamada/golpe de aviso</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>acuerdo de vecindad con llamada golpe de aviso</t>
-        </is>
-      </c>
+          <t>Regulador de carga MPPT 60A</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -1481,13 +1453,525 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Energía solar: el sol es tu generador</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Cableado y protección solar (cables UV, MC4, fusibles, interruptores DC)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Baterías de litio LFP: almacena tu energía</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Batería litio LFP 200Ah (48V) — 9,6 kWh</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Baterías de litio LFP: almacena tu energía</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Segunda batería LFP 200Ah (sistema paralelo) — 19,2 kWh</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Baterías de litio LFP: almacena tu energía</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Caja de fusibles y distribución DC para baterías</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SAI (UPS): conmutación instantánea</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SAI (UPS) 3000VA-5000VA online doble conversión</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SAI (UPS): conmutación instantánea</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SAI 1500VA online (equipos críticos individuales)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Generador: respaldo cuando no hay sol</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Generador inverter 2000-3000W (gasolina o gas)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Generador: respaldo cuando no hay sol</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Depósito ampliado o conexión a gas natural</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Conservación de alimentos sin red</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Nevera/congeladora solar 12V/220V (compresor)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Conservación de alimentos sin red</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Acumuladores de frío congelables (pack de 6)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Iluminación y seguridad perimetral</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Set de 10 luminarias LED solares de jardín</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Iluminación y seguridad perimetral</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Cámara de seguridad solar 4G con batería</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
           <t>sin candidato verificado</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Conectividad: Starlink y redundancia</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Terminal Starlink Gen 3 (residencial / móvil)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>propuesta</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Conectividad: Starlink y redundancia</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Router 4G/5G industrial con dual SIM y antenas externas</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>sin candidato verificado</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Conectividad: Starlink y redundancia</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Messenger satelital (Garmin inReach Mini 3)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>sin candidato verificado</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>kit-kit-profesional</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Conectividad: Starlink y redundancia</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Extensor WiFi de largo alcance + antena direccional</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>sin candidato verificado</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A1:L45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>